<commit_message>
Preping ecopath models and biomass estimates for BDSC
</commit_message>
<xml_diff>
--- a/MattsRpath/RPath_parameterdraftlist.xlsx
+++ b/MattsRpath/RPath_parameterdraftlist.xlsx
@@ -5,21 +5,22 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cawater-my.sharepoint.com/personal/rosemary_hartman_water_ca_gov/Documents/food webs/FoodwebModel/MattsRpath/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rhartman\OneDrive - California Department of Water Resources\food webs\FoodwebModel\MattsRpath\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="556" documentId="8_{6BDD44C6-9D4B-4160-A4C5-B8CC2CF85AEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6490C885-7DB3-4181-AF35-6514DD7C1C59}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F248DE40-DD1D-4563-B2F2-F5B871348457}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00E913D7-4E82-4E87-9828-59006E2DA130}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00E913D7-4E82-4E87-9828-59006E2DA130}"/>
   </bookViews>
   <sheets>
     <sheet name="Matt's origional" sheetId="1" r:id="rId1"/>
-    <sheet name="biomassPerHabitat" sheetId="7" r:id="rId2"/>
-    <sheet name="testparams" sheetId="5" r:id="rId3"/>
+    <sheet name="testparams" sheetId="5" r:id="rId2"/>
+    <sheet name="InsectPlaceholder" sheetId="7" r:id="rId3"/>
     <sheet name="dietmatrix" sheetId="6" r:id="rId4"/>
     <sheet name="New params" sheetId="2" r:id="rId5"/>
-    <sheet name="StableIsotopDiets" sheetId="3" r:id="rId6"/>
-    <sheet name="Schroeteretal2015" sheetId="4" r:id="rId7"/>
+    <sheet name="primary producers" sheetId="8" r:id="rId6"/>
+    <sheet name="StableIsotopDiets" sheetId="3" r:id="rId7"/>
+    <sheet name="Schroeteretal2015" sheetId="4" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -173,6 +174,24 @@
 <file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={2253C964-8575-457F-84DF-2AEB9F95108B}</author>
+  </authors>
+  <commentList>
+    <comment ref="C8" authorId="0" shapeId="0" xr:uid="{2253C964-8575-457F-84DF-2AEB9F95108B}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    0.400 based on Zierdt Smith. Used calcs from Young et al 2018</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
     <author>tc={04240FD7-3159-44A0-9F39-44A4916A7AC7}</author>
     <author>tc={578F8387-4BAD-482C-B1E9-88C2D9EA758C}</author>
     <author>tc={0F7BB635-BF16-4204-AAE2-648861855766}</author>
@@ -296,7 +315,7 @@
 </comments>
 </file>
 
-<file path=xl/comments3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={0EBA0974-1903-4504-A4F0-A966FA96781C}</author>
@@ -315,7 +334,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="700" uniqueCount="178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="712" uniqueCount="193">
   <si>
     <t>Site</t>
   </si>
@@ -812,43 +831,88 @@
     <t>Fishing.disc</t>
   </si>
   <si>
+    <t>PredatoryCopepods</t>
+  </si>
+  <si>
+    <t>OtherCopepods</t>
+  </si>
+  <si>
+    <t>Limnoithona</t>
+  </si>
+  <si>
+    <t>FAV</t>
+  </si>
+  <si>
+    <t>Confluence</t>
+  </si>
+  <si>
+    <t>Chironomids</t>
+  </si>
+  <si>
     <t>Import</t>
   </si>
   <si>
-    <t>PredatoryCopepods</t>
-  </si>
-  <si>
-    <t>OtherCopepods</t>
-  </si>
-  <si>
-    <t>Limnoithona</t>
-  </si>
-  <si>
-    <t>Emergent</t>
-  </si>
-  <si>
-    <t>FAV</t>
-  </si>
-  <si>
-    <t>Water</t>
-  </si>
-  <si>
-    <t>Soil/mudflat</t>
-  </si>
-  <si>
-    <t>Confluence</t>
-  </si>
-  <si>
-    <t>Grizzly</t>
-  </si>
-  <si>
-    <t>Decker</t>
-  </si>
-  <si>
-    <t>Webb</t>
-  </si>
-  <si>
-    <t>x</t>
+    <t>Habitat</t>
+  </si>
+  <si>
+    <t>Open Water</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>miller and fiji</t>
+  </si>
+  <si>
+    <t>Matt's number</t>
+  </si>
+  <si>
+    <t>Conrad et al 2016, median 250 g/m4 dry mass. .25kg/m2 * 1000ha/m2*10 gWW/gDW. Conrad cite Santos 2011 for DW;WW conversion but I couldn't find it</t>
+  </si>
+  <si>
+    <t>Marineau et al 40gDW/.25m2 quadrat. 0.04kg*4*10000*10</t>
+  </si>
+  <si>
+    <t>just making this up</t>
+  </si>
+  <si>
+    <t>This is producitivty values from Cloern et al, not sure how it really applies to standing biomass</t>
+  </si>
+  <si>
+    <t>This is producitivty values from Cloern et al, not sure how it really applies to standing biomass. 44 g/m2/year</t>
+  </si>
+  <si>
+    <t>Gammarids</t>
+  </si>
+  <si>
+    <t>Corophiids</t>
+  </si>
+  <si>
+    <t>Gammaroids</t>
+  </si>
+  <si>
+    <t>Decker/Webb</t>
+  </si>
+  <si>
+    <t>Grizzly Bay</t>
+  </si>
+  <si>
+    <t>Cache Slough</t>
+  </si>
+  <si>
+    <t>Inside</t>
+  </si>
+  <si>
+    <t>Outside</t>
+  </si>
+  <si>
+    <t>Damselflies</t>
+  </si>
+  <si>
+    <t>Damselfliess</t>
+  </si>
+  <si>
+    <t>InsideOutside</t>
   </si>
 </sst>
 </file>
@@ -948,7 +1012,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -987,9 +1051,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1622,6 +1683,14 @@
 
 <file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="C8" dT="2023-05-17T20:32:54.88" personId="{FF688BB4-8F7E-4979-94D0-6877041B0073}" id="{2253C964-8575-457F-84DF-2AEB9F95108B}">
+    <text>0.400 based on Zierdt Smith. Used calcs from Young et al 2018</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
+<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="H1" dT="2023-03-28T23:48:01.57" personId="{FF688BB4-8F7E-4979-94D0-6877041B0073}" id="{04240FD7-3159-44A0-9F39-44A4916A7AC7}">
     <text>Production/Biomass</text>
   </threadedComment>
@@ -1664,7 +1733,7 @@
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/threadedComments/threadedComment4.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <threadedComment ref="B11" dT="2026-07-02T16:57:49.31" personId="{3A46231C-F56C-4F36-B3C0-70549FD48C92}" id="{0EBA0974-1903-4504-A4F0-A966FA96781C}">
     <text>Do we want predatory insects from Young et al?</text>
@@ -3712,470 +3781,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8675226-D191-481E-B450-083710A2914C}">
-  <dimension ref="A1:G46"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="2" max="2" width="23.26953125" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1" t="s">
-        <v>169</v>
-      </c>
-      <c r="D1" t="s">
-        <v>170</v>
-      </c>
-      <c r="E1" t="s">
-        <v>78</v>
-      </c>
-      <c r="F1" t="s">
-        <v>171</v>
-      </c>
-      <c r="G1" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
-        <v>113</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
-        <v>113</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4">
-        <v>0</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" t="s">
-        <v>113</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" t="s">
-        <v>113</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>0</v>
-      </c>
-      <c r="E7">
-        <v>0</v>
-      </c>
-      <c r="F7" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A8" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
-        <v>113</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" t="s">
-        <v>113</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" t="s">
-        <v>173</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
-        <v>173</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
-        <v>173</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" t="s">
-        <v>173</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A15" t="s">
-        <v>173</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
-        <v>173</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
-        <v>173</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>173</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
-        <v>173</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A20" t="s">
-        <v>174</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A21" t="s">
-        <v>174</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
-        <v>174</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A23" t="s">
-        <v>174</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A24" t="s">
-        <v>174</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A25" t="s">
-        <v>174</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A26" t="s">
-        <v>174</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A27" t="s">
-        <v>174</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
-        <v>174</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
-        <v>175</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A30" t="s">
-        <v>175</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A31" t="s">
-        <v>175</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A32" t="s">
-        <v>175</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
-        <v>175</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
-        <v>175</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>175</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
-        <v>175</v>
-      </c>
-      <c r="B36" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>175</v>
-      </c>
-      <c r="B37" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A38" t="s">
-        <v>176</v>
-      </c>
-      <c r="B38" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A39" t="s">
-        <v>176</v>
-      </c>
-      <c r="B39" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>176</v>
-      </c>
-      <c r="B40" s="3" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A41" t="s">
-        <v>176</v>
-      </c>
-      <c r="B41" s="3" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A42" t="s">
-        <v>176</v>
-      </c>
-      <c r="B42" s="3" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>176</v>
-      </c>
-      <c r="B43" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A44" t="s">
-        <v>176</v>
-      </c>
-      <c r="B44" s="3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>176</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A46" t="s">
-        <v>176</v>
-      </c>
-      <c r="B46" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D90776B-D387-4A99-8EF1-CBCC147CD9BF}">
-  <dimension ref="A1:M17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D90776B-D387-4A99-8EF1-CBCC147CD9BF}">
+  <dimension ref="A1:M18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="23.26953125" bestFit="1" customWidth="1"/>
@@ -4235,7 +3842,7 @@
         <v>0</v>
       </c>
       <c r="C2" s="3">
-        <v>114.449</v>
+        <v>114</v>
       </c>
       <c r="D2" t="s">
         <v>156</v>
@@ -4247,7 +3854,7 @@
         <v>10</v>
       </c>
       <c r="G2" s="3">
-        <f t="shared" ref="G2:G10" si="0">E2/F2</f>
+        <f t="shared" ref="G2:G11" si="0">E2/F2</f>
         <v>0.12</v>
       </c>
       <c r="H2">
@@ -4273,72 +3880,189 @@
       <c r="A3" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="L3" s="3"/>
-      <c r="M3" s="3"/>
+      <c r="B3" s="3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="3">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E3" s="5">
+        <v>3</v>
+      </c>
+      <c r="F3" s="3">
+        <v>10</v>
+      </c>
+      <c r="G3" s="3">
+        <f t="shared" ref="G3" si="1">E3/F3</f>
+        <v>0.3</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0.2</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3" s="3">
+        <v>0</v>
+      </c>
+      <c r="M3" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="L4" s="3"/>
-      <c r="M4" s="3"/>
+        <v>165</v>
+      </c>
+      <c r="B4" s="3">
+        <v>0</v>
+      </c>
+      <c r="C4" s="3">
+        <v>0.2</v>
+      </c>
+      <c r="D4" t="s">
+        <v>156</v>
+      </c>
+      <c r="E4" s="5">
+        <v>30</v>
+      </c>
+      <c r="F4" s="3">
+        <v>100</v>
+      </c>
+      <c r="G4" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0.2</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>1</v>
+      </c>
+      <c r="L4" s="3">
+        <v>0</v>
+      </c>
+      <c r="M4" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="3"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
-      <c r="L5" s="3"/>
-      <c r="M5" s="3"/>
+        <v>166</v>
+      </c>
+      <c r="B5" s="3">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3">
+        <v>15</v>
+      </c>
+      <c r="D5" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" s="5">
+        <v>50</v>
+      </c>
+      <c r="F5" s="3">
+        <v>100</v>
+      </c>
+      <c r="G5" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0.2</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5" s="3">
+        <v>0</v>
+      </c>
+      <c r="M5" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
-      <c r="L6" s="3"/>
-      <c r="M6" s="3"/>
+        <v>167</v>
+      </c>
+      <c r="B6" s="3">
+        <v>0</v>
+      </c>
+      <c r="C6" s="3">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>156</v>
+      </c>
+      <c r="E6" s="5">
+        <v>50</v>
+      </c>
+      <c r="F6" s="3">
+        <v>100</v>
+      </c>
+      <c r="G6" s="3">
+        <v>0.5</v>
+      </c>
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0.2</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="L6" s="3">
+        <v>0</v>
+      </c>
+      <c r="M6" s="3">
+        <v>0</v>
+      </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7" s="3" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="B7" s="3">
         <v>0</v>
       </c>
       <c r="C7" s="3">
-        <v>5878.5240000000003</v>
+        <v>1</v>
       </c>
       <c r="D7" t="s">
         <v>156</v>
       </c>
       <c r="E7" s="5">
-        <v>3</v>
+        <v>57.3</v>
       </c>
       <c r="F7" s="3">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="G7" s="3">
-        <f t="shared" si="0"/>
-        <v>0.6</v>
+        <f>E7/F7</f>
+        <v>0.57299999999999995</v>
       </c>
       <c r="H7">
         <v>0</v>
@@ -4361,13 +4085,13 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8" s="3" t="s">
-        <v>62</v>
+        <v>182</v>
       </c>
       <c r="B8" s="3">
         <v>0</v>
       </c>
       <c r="C8" s="3">
-        <v>11.471</v>
+        <v>5878.5240000000003</v>
       </c>
       <c r="D8" t="s">
         <v>156</v>
@@ -4403,13 +4127,13 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9" s="3" t="s">
-        <v>64</v>
+        <v>183</v>
       </c>
       <c r="B9" s="3">
         <v>0</v>
       </c>
       <c r="C9" s="3">
-        <v>2934.8919999999998</v>
+        <v>11.471</v>
       </c>
       <c r="D9" t="s">
         <v>156</v>
@@ -4445,26 +4169,26 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10" s="3" t="s">
-        <v>69</v>
+        <v>170</v>
       </c>
       <c r="B10" s="3">
         <v>0</v>
       </c>
-      <c r="C10" s="3">
-        <v>0.218</v>
+      <c r="C10">
+        <v>25</v>
       </c>
       <c r="D10" t="s">
         <v>156</v>
       </c>
       <c r="E10" s="5">
-        <v>57.3</v>
+        <v>10</v>
       </c>
       <c r="F10" s="3">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="G10" s="3">
         <f t="shared" si="0"/>
-        <v>0.57299999999999995</v>
+        <v>2</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -4487,31 +4211,32 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11" s="3" t="s">
-        <v>78</v>
+        <v>190</v>
       </c>
       <c r="B11" s="3">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="3">
-        <v>874</v>
-      </c>
-      <c r="D11" s="3">
-        <v>0.1</v>
+        <v>0.01</v>
+      </c>
+      <c r="D11" t="s">
+        <v>156</v>
       </c>
       <c r="E11" s="5">
-        <v>220.005</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>156</v>
+        <v>3</v>
+      </c>
+      <c r="F11" s="3">
+        <v>5</v>
+      </c>
+      <c r="G11" s="3">
+        <f t="shared" si="0"/>
+        <v>0.6</v>
       </c>
       <c r="H11">
         <v>0</v>
       </c>
-      <c r="I11" s="3">
-        <v>0.9</v>
+      <c r="I11">
+        <v>0.2</v>
       </c>
       <c r="J11">
         <v>0</v>
@@ -4528,19 +4253,19 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="3" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B12" s="3">
         <v>1</v>
       </c>
       <c r="C12" s="3">
-        <v>213.91</v>
+        <v>874</v>
       </c>
       <c r="D12" s="3">
-        <v>0.8</v>
+        <v>0.1</v>
       </c>
       <c r="E12" s="5">
-        <v>209.87799999999999</v>
+        <v>220.005</v>
       </c>
       <c r="F12" s="3" t="s">
         <v>156</v>
@@ -4552,7 +4277,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="3">
-        <v>0.2</v>
+        <v>0.9</v>
       </c>
       <c r="J12">
         <v>0</v>
@@ -4569,19 +4294,19 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B13" s="3">
         <v>1</v>
       </c>
       <c r="C13" s="3">
-        <v>160.928</v>
+        <v>213.91</v>
       </c>
       <c r="D13" s="3">
         <v>0.8</v>
       </c>
       <c r="E13" s="5">
-        <v>133.22499999999999</v>
+        <v>209.87799999999999</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>156</v>
@@ -4610,19 +4335,19 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B14" s="3">
         <v>1</v>
       </c>
       <c r="C14" s="3">
-        <v>16000</v>
+        <v>160.928</v>
       </c>
       <c r="D14" s="3">
-        <v>0.05</v>
+        <v>0.8</v>
       </c>
       <c r="E14" s="5">
-        <v>2</v>
+        <v>133.22499999999999</v>
       </c>
       <c r="F14" s="3" t="s">
         <v>156</v>
@@ -4634,7 +4359,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="3">
-        <v>0.9</v>
+        <v>0.2</v>
       </c>
       <c r="J14">
         <v>0</v>
@@ -4651,19 +4376,19 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B15" s="3">
         <v>1</v>
       </c>
       <c r="C15" s="3">
-        <v>200</v>
+        <v>2000</v>
       </c>
       <c r="D15" s="3">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="E15" s="5">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F15" s="3" t="s">
         <v>156</v>
@@ -4692,19 +4417,19 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="3" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B16" s="3">
-        <v>2</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>156</v>
-      </c>
-      <c r="E16" s="5" t="s">
-        <v>156</v>
+        <v>1</v>
+      </c>
+      <c r="C16" s="3">
+        <v>15</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0.1</v>
+      </c>
+      <c r="E16" s="5">
+        <v>6</v>
       </c>
       <c r="F16" s="3" t="s">
         <v>156</v>
@@ -4713,7 +4438,7 @@
         <v>156</v>
       </c>
       <c r="H16">
-        <v>1000</v>
+        <v>0</v>
       </c>
       <c r="I16" s="3">
         <v>0.9</v>
@@ -4733,10 +4458,10 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
-        <v>163</v>
+        <v>87</v>
       </c>
       <c r="B17" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C17" s="3" t="s">
         <v>156</v>
@@ -4753,11 +4478,11 @@
       <c r="G17" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="H17" t="s">
-        <v>156</v>
-      </c>
-      <c r="I17" s="3" t="s">
-        <v>156</v>
+      <c r="H17">
+        <v>1000</v>
+      </c>
+      <c r="I17" s="3">
+        <v>0.9</v>
       </c>
       <c r="J17">
         <v>0</v>
@@ -4772,20 +4497,402 @@
         <v>0</v>
       </c>
     </row>
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A18" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="B18" s="3">
+        <v>3</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="E18" s="5" t="s">
+        <v>156</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="H18" t="s">
+        <v>156</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="J18">
+        <v>0</v>
+      </c>
+      <c r="K18">
+        <v>1</v>
+      </c>
+      <c r="L18" s="3">
+        <v>0</v>
+      </c>
+      <c r="M18" s="3">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B8675226-D191-481E-B450-083710A2914C}">
+  <dimension ref="A1:D45"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.54296875" customWidth="1"/>
+    <col min="3" max="3" width="23.26953125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B1" t="s">
+        <v>192</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="D1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>187</v>
+      </c>
+      <c r="B2" t="s">
+        <v>188</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D2">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>169</v>
+      </c>
+      <c r="B3" t="s">
+        <v>188</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D3">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>185</v>
+      </c>
+      <c r="B4" t="s">
+        <v>188</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D4">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>187</v>
+      </c>
+      <c r="B6" t="s">
+        <v>189</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>169</v>
+      </c>
+      <c r="B7" t="s">
+        <v>189</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>185</v>
+      </c>
+      <c r="B8" t="s">
+        <v>189</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D8">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B9" t="s">
+        <v>189</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>187</v>
+      </c>
+      <c r="B10" t="s">
+        <v>188</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D10">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>169</v>
+      </c>
+      <c r="B11" t="s">
+        <v>188</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D11">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>185</v>
+      </c>
+      <c r="B12" t="s">
+        <v>188</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D12">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>186</v>
+      </c>
+      <c r="B13" t="s">
+        <v>188</v>
+      </c>
+      <c r="C13" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>187</v>
+      </c>
+      <c r="B14" t="s">
+        <v>189</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D14">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>169</v>
+      </c>
+      <c r="B15" t="s">
+        <v>189</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D15">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>185</v>
+      </c>
+      <c r="B16" t="s">
+        <v>189</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D16">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>186</v>
+      </c>
+      <c r="B17" t="s">
+        <v>189</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="D17">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C18" s="3"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C19" s="3"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C20" s="3"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C21" s="3"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C22" s="3"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C23" s="3"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C24" s="3"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C25" s="3"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C26" s="3"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C27" s="3"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C28" s="3"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C29" s="3"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C30" s="3"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C31" s="3"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="C32" s="3"/>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C33" s="3"/>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C34" s="3"/>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C35" s="3"/>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C36" s="3"/>
+    </row>
+    <row r="37" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C37" s="3"/>
+    </row>
+    <row r="38" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C38" s="3"/>
+    </row>
+    <row r="39" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C39" s="3"/>
+    </row>
+    <row r="40" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C40" s="3"/>
+    </row>
+    <row r="41" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C41" s="3"/>
+    </row>
+    <row r="42" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C42" s="3"/>
+    </row>
+    <row r="43" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C43" s="3"/>
+    </row>
+    <row r="44" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C44" s="3"/>
+    </row>
+    <row r="45" spans="3:3" x14ac:dyDescent="0.35">
+      <c r="C45" s="3"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:G45">
+    <sortCondition ref="C2:C45"/>
+    <sortCondition ref="A2:A45"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8507B781-AD72-4DC8-A4BE-7CF19625E49F}">
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:R18"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="21.1796875" style="15" customWidth="1"/>
     <col min="3" max="3" width="13.81640625" customWidth="1"/>
     <col min="4" max="4" width="15.54296875" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="21.1796875" customWidth="1"/>
     <col min="6" max="8" width="12.81640625" customWidth="1"/>
     <col min="9" max="9" width="11.7265625" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
@@ -4796,7 +4903,7 @@
     <col min="16" max="16" width="15" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>96</v>
       </c>
@@ -4804,124 +4911,147 @@
         <v>55</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>59</v>
+        <v>143</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>60</v>
+        <v>165</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>62</v>
+        <v>166</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>92</v>
+        <v>167</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>69</v>
+        <v>184</v>
       </c>
       <c r="I1" s="3" t="s">
-        <v>71</v>
+        <v>183</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>74</v>
+        <v>170</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="L1" s="16" t="s">
+        <v>190</v>
+      </c>
+      <c r="L1" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="M1" s="16" t="s">
+      <c r="M1" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="N1" s="16" t="s">
+      <c r="N1" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="O1" s="16" t="s">
+      <c r="O1" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="P1" s="16" t="s">
+      <c r="P1" s="3" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="16" t="s">
+      <c r="Q1" s="3"/>
+      <c r="R1" s="3"/>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3" s="16" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="C4">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A3" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A5" s="3" t="s">
+        <v>166</v>
+      </c>
+      <c r="C5">
+        <v>0.05</v>
+      </c>
+      <c r="D5">
+        <v>0.5</v>
+      </c>
+      <c r="K5">
         <v>0.1</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" s="16" t="s">
-        <v>62</v>
-      </c>
-      <c r="C5">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6" s="16" t="s">
-        <v>92</v>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>167</v>
       </c>
       <c r="C6">
         <v>0.1</v>
       </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A7" s="16" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
+      <c r="D6">
+        <v>0.5</v>
+      </c>
+      <c r="K6">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A7" s="3" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A9" s="16" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A10" s="16" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A11" s="16" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A12" s="16" t="s">
+      <c r="K7">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A8" s="3" t="s">
+        <v>184</v>
+      </c>
+      <c r="K8">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>183</v>
+      </c>
+      <c r="K9">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A10" s="3" t="s">
+        <v>170</v>
+      </c>
+      <c r="K10">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A11" s="3" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A12" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="C12">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A13" s="16" t="s">
+      <c r="J12">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A13" s="3" t="s">
         <v>81</v>
       </c>
       <c r="B13">
         <v>0.8</v>
       </c>
-      <c r="D13">
-        <v>0.1</v>
+      <c r="C13">
+        <v>0.6</v>
       </c>
       <c r="E13">
         <v>0.4</v>
@@ -4930,27 +5060,24 @@
         <v>0.25</v>
       </c>
       <c r="G13">
-        <v>0.16</v>
+        <v>0.6</v>
       </c>
       <c r="H13">
-        <v>0.57999999999999996</v>
+        <v>0.3</v>
       </c>
       <c r="I13">
         <v>0.63</v>
       </c>
       <c r="J13">
-        <v>0.63</v>
+        <v>0.3</v>
       </c>
       <c r="K13">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A14" s="16" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A14" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="D14">
-        <v>0.15</v>
       </c>
       <c r="E14">
         <v>0.08</v>
@@ -4968,37 +5095,31 @@
         <v>3.6999999999999998E-2</v>
       </c>
       <c r="J14">
-        <v>3.6999999999999998E-2</v>
+        <v>0.2</v>
       </c>
       <c r="K14">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A15" s="16" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A15" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="C15">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A16" s="16" t="s">
+    </row>
+    <row r="16" spans="1:18" x14ac:dyDescent="0.35">
+      <c r="A16" s="3" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="3" t="s">
         <v>87</v>
       </c>
       <c r="B17">
         <v>0.2</v>
       </c>
       <c r="C17">
-        <v>0.3</v>
-      </c>
-      <c r="D17">
-        <v>0.75</v>
+        <v>0.25</v>
       </c>
       <c r="E17">
         <f>1-(E13+E14)</f>
@@ -5010,28 +5131,28 @@
       </c>
       <c r="G17">
         <f>1-(G13+G14)</f>
-        <v>0.73</v>
+        <v>0.29000000000000004</v>
       </c>
       <c r="H17">
         <f t="shared" ref="H17:I17" si="0">1-(H13+H14)</f>
-        <v>0.38</v>
+        <v>0.66</v>
       </c>
       <c r="I17">
         <f t="shared" si="0"/>
         <v>0.33299999999999996</v>
       </c>
       <c r="J17">
-        <f t="shared" ref="J17:K17" si="1">1-(J13+J14)</f>
-        <v>0.33299999999999996</v>
+        <f>1-(J13+J14+J12)</f>
+        <v>0.19999999999999996</v>
       </c>
       <c r="K17">
-        <f t="shared" si="1"/>
-        <v>0.5</v>
+        <f>1-(SUM(K2:K14))</f>
+        <v>0.30000000000000004</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="15" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
   </sheetData>
@@ -7309,6 +7430,294 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A8F03784-4B6F-4B20-972D-79163B018065}">
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="12.453125" customWidth="1"/>
+    <col min="2" max="2" width="20.6328125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D1" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C2">
+        <v>50</v>
+      </c>
+      <c r="D2" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C3">
+        <v>50</v>
+      </c>
+      <c r="D3" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>168</v>
+      </c>
+      <c r="B4" t="s">
+        <v>81</v>
+      </c>
+      <c r="C4">
+        <v>50</v>
+      </c>
+      <c r="D4" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C5" s="3">
+        <v>213.91</v>
+      </c>
+      <c r="D5" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C6" s="3">
+        <f>1.6*10000</f>
+        <v>16000</v>
+      </c>
+      <c r="D6" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>168</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>173</v>
+      </c>
+      <c r="B9" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B10" t="s">
+        <v>78</v>
+      </c>
+      <c r="C10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C11">
+        <f>0.25*10000*10</f>
+        <v>25000</v>
+      </c>
+      <c r="D11" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>168</v>
+      </c>
+      <c r="B12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>173</v>
+      </c>
+      <c r="B13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A14" t="s">
+        <v>126</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C14">
+        <f>0.044*10000</f>
+        <v>440</v>
+      </c>
+      <c r="D14" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B15" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C15">
+        <f>0.024*10000</f>
+        <v>240</v>
+      </c>
+      <c r="D15" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>168</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C16">
+        <f>0.015*10000</f>
+        <v>150</v>
+      </c>
+      <c r="D16" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A17" t="s">
+        <v>173</v>
+      </c>
+      <c r="B17" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="C17">
+        <f>0.04*10000</f>
+        <v>400</v>
+      </c>
+      <c r="D17" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A18" t="s">
+        <v>126</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C18">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A20" t="s">
+        <v>168</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20">
+        <f>0.04*4*10000*10</f>
+        <v>16000</v>
+      </c>
+      <c r="D20" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A21" t="s">
+        <v>173</v>
+      </c>
+      <c r="B21" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C21">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{885072BE-048E-4823-9B10-4C85A9AD3529}">
   <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -7867,7 +8276,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{570365D2-CF0E-4D4C-9C66-9B0194DA64C1}">
   <dimension ref="A1:J23"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>